<commit_message>
fix: cells with the default style keep the default font and border when a loaded stylesheet's first font or border is another (#792)
The styles writer mapped the default style to font 0, fill 0 and border 0. A loaded stylesheet keeps its order, so index 0 can hold another font: cells in Calibri 11 were saved with the file's first font, Arial 20. The default style's ids are now looked up like every other style's, and it is written only when the stylesheet is new or something uses it, so a loaded file gains no unused cellXf. The UsingPhonetics reference file recorded the bug: its cell pointed at the 8 pt phonetic font.
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/Styles/UsingPhonetics.xlsx
+++ b/XLibur.Tests/Resource/Examples/Styles/UsingPhonetics.xlsx
@@ -86,12 +86,12 @@
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
   <x:cellXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>

</xml_diff>

<commit_message>
fix: the styles part is written before the shared strings, so phoneticPr/@fontId names the phonetic font and the default font stays fonts[0] (#801, #802)
The shared strings registered each phonetic font in SaveContext.SharedFonts before the styles part gave fonts their ids, so phoneticPr/@fontId was always 0 and, in a new workbook, the phonetic font took index 0 ahead of the default font. The styles part now registers the phonetic fonts of every text in use, after the default font and the styles' fonts, and is written first; the text writers only look the id up. An inline text's phonetic font is now written to the styles part too.

Closes #801

Closes #802
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/Styles/UsingPhonetics.xlsx
+++ b/XLibur.Tests/Resource/Examples/Styles/UsingPhonetics.xlsx
@@ -45,14 +45,14 @@
   <x:fonts count="2">
     <x:font>
       <x:vertAlign val="baseline"/>
-      <x:sz val="8"/>
+      <x:sz val="11"/>
       <x:color rgb="FF000000"/>
       <x:name val="Calibri"/>
       <x:family val="2"/>
     </x:font>
     <x:font>
       <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
+      <x:sz val="8"/>
       <x:color rgb="FF000000"/>
       <x:name val="Calibri"/>
       <x:family val="2"/>
@@ -86,12 +86,12 @@
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
   <x:cellXfs count="1">
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>

</xml_diff>